<commit_message>
Fix eda + record
</commit_message>
<xml_diff>
--- a/Challeng_1_Titanic_Final/process/exps/record.xlsx
+++ b/Challeng_1_Titanic_Final/process/exps/record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dai_hoc\nam3\HK5\ML\LAB_GROUP\Challeng_1_Titanic_Final\process\exps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F398DB-B452-4923-B2E2-59B5D6AA5E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE2545C-9F2C-48C1-AD94-64B620D8239F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="112">
   <si>
     <t>Xử lý missing value</t>
   </si>
@@ -318,6 +318,48 @@
   </si>
   <si>
     <t>KNN với biến 'Pclass'</t>
+  </si>
+  <si>
+    <t>Voting</t>
+  </si>
+  <si>
+    <t>Stacking</t>
+  </si>
+  <si>
+    <t>Blending</t>
+  </si>
+  <si>
+    <t>Weighted Average</t>
+  </si>
+  <si>
+    <t>0.8224</t>
+  </si>
+  <si>
+    <t>0.9329</t>
+  </si>
+  <si>
+    <t>0.79426</t>
+  </si>
+  <si>
+    <t>0.79428</t>
+  </si>
+  <si>
+    <t>0.8732</t>
+  </si>
+  <si>
+    <t>0.8243</t>
+  </si>
+  <si>
+    <t>0.9327</t>
+  </si>
+  <si>
+    <t>0.8743</t>
+  </si>
+  <si>
+    <t>0.8245</t>
+  </si>
+  <si>
+    <t>0.9318</t>
   </si>
 </sst>
 </file>
@@ -573,6 +615,21 @@
     <xf numFmtId="3" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -603,21 +660,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -627,7 +669,7 @@
     <xf numFmtId="3" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -949,17 +991,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="24" t="s">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="D1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -1059,10 +1101,10 @@
     </row>
     <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="23"/>
+      <c r="B8" s="28"/>
     </row>
     <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
@@ -1141,17 +1183,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="24" t="s">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="D1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="26"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="31"/>
     </row>
     <row r="2" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -1257,10 +1299,10 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="23"/>
+      <c r="B8" s="28"/>
     </row>
     <row r="9" spans="1:8" s="7" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
@@ -1346,17 +1388,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="E1" s="24" t="s">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="E1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
     </row>
     <row r="2" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -1382,10 +1424,10 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="26" t="s">
         <v>96</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -1405,10 +1447,10 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="26" t="s">
         <v>96</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -1464,11 +1506,11 @@
       </c>
     </row>
     <row r="8" spans="1:9" s="19" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="29"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="34"/>
     </row>
     <row r="9" spans="1:9" s="18" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
@@ -1577,17 +1619,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="E1" s="30" t="s">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="E1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
     </row>
     <row r="2" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -1744,24 +1786,24 @@
       </c>
     </row>
     <row r="13" spans="1:9" s="7" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="34">
+      <c r="C13" s="23">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="7" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="34">
+      <c r="C14" s="23">
         <v>1</v>
       </c>
     </row>
@@ -1836,17 +1878,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="E1" s="30" t="s">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="E1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
     </row>
     <row r="2" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -1872,10 +1914,10 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="26" t="s">
         <v>97</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -1947,18 +1989,62 @@
       <c r="B6" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E7" s="6"/>
+      <c r="E6" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E7" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="32"/>
-    </row>
-    <row r="9" spans="1:9" s="7" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="36"/>
+      <c r="C8" s="40"/>
+      <c r="E8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="7" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
         <v>2</v>
       </c>
@@ -1967,6 +2053,21 @@
       </c>
       <c r="C9" s="17" t="s">
         <v>33</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="7" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1992,57 +2093,57 @@
       </c>
     </row>
     <row r="12" spans="1:9" s="7" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="36">
+      <c r="C12" s="25">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" s="7" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="35" t="s">
+      <c r="A13" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="36">
+      <c r="C13" s="25">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="7" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="25">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="7" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="34">
+      <c r="C15" s="23">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:9" s="7" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C16" s="34">
+      <c r="C16" s="23">
         <v>1</v>
       </c>
     </row>
@@ -2091,35 +2192,35 @@
       </c>
     </row>
     <row r="21" spans="1:3" s="7" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="35" t="s">
+      <c r="A21" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="36">
+      <c r="C21" s="25">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="18" x14ac:dyDescent="0.3">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="B22" s="35" t="s">
+      <c r="B22" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="36">
+      <c r="C22" s="25">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="35" t="s">
+      <c r="A23" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="35" t="s">
+      <c r="B23" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="36">
+      <c r="C23" s="25">
         <v>0</v>
       </c>
     </row>

</xml_diff>